<commit_message>
Usar un parametro de Power Query para la ruta y evitar Formula.Firewall
La consulta Ventas referenciaba la consulta RutaDatos y ademas accedia a un
origen externo con File.Contents en el mismo paso, que es la condicion que
dispara el error Formula.Firewall al actualizar.

RutaDatos pasa a ser un parametro real (IsParameterQuery), que el motor
resuelve como valor literal antes de evaluar la consulta y por lo tanto no
cuenta como referencia entre consultas.

- Nuevo control: ningun File.Contents puede tener la ruta hardcodeada
- Pasos A y B de la hoja PASOS_EN_EXCEL reescritos para el parametro
- README del repositorio: se agrega el checkpoint de modelado BI

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RW3rLtX7kWM4MbF8vmj54N
</commit_message>
<xml_diff>
--- a/checkpoint-modelo-bi/PreEntrega_ModeloBI_MurphyLleyton.xlsx
+++ b/checkpoint-modelo-bi/PreEntrega_ModeloBI_MurphyLleyton.xlsx
@@ -941,7 +941,14 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Esta celda se llama RutaDatos. La consulta del mismo nombre la lee con Excel.CurrentWorkbook() y las otras cuatro consultas la concatenan con el nombre de archivo. Para mover el proyecto de carpeta alcanza con editar esta celda y actualizar; no hay que tocar ninguna consulta.</t>
+          <t>Este es el valor que hay que cargar en el parametro RutaDatos de Power Query (Inicio &gt; Administrar parametros). Las cuatro consultas lo concatenan con el nombre de archivo, asi que la ruta esta escrita una sola vez: mover el proyecto de carpeta es editar el parametro, no las consultas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Se usa un parametro y no una celda leida con Excel.CurrentWorkbook() para no disparar el error Formula.Firewall, que aparece cuando una consulta referencia a otra y ademas accede a un origen externo en el mismo paso.</t>
         </is>
       </c>
     </row>
@@ -965,12 +972,13 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A6"/>
     <mergeCell ref="A5"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
@@ -2317,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B255"/>
+  <dimension ref="B2:B273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2348,7 +2356,7 @@
     <row r="6">
       <c r="B6" s="55" t="inlineStr">
         <is>
-          <t>// Consulta: RutaDatos   (parametro)</t>
+          <t>// Parametro: RutaDatos</t>
         </is>
       </c>
     </row>
@@ -2362,21 +2370,21 @@
     <row r="8">
       <c r="B8" s="55" t="inlineStr">
         <is>
-          <t>// Evita la ruta de origen "hardcodeada". En lugar de escribir C:\Users\...\datos</t>
+          <t>// Resuelve el problema de la ruta de origen "hardcodeada": en lugar de repetir</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="55" t="inlineStr">
         <is>
-          <t>// dentro de cada consulta, el path se lee desde la celda con nombre RutaDatos</t>
+          <t>// C:\...\datos dentro de cada consulta, el path vive en un unico lugar y las</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="55" t="inlineStr">
         <is>
-          <t>// de la hoja Config del propio libro.</t>
+          <t>// cuatro consultas lo concatenan con el nombre de archivo.</t>
         </is>
       </c>
     </row>
@@ -2390,327 +2398,339 @@
     <row r="12">
       <c r="B12" s="55" t="inlineStr">
         <is>
-          <t>// Resultado: el evaluador puede mover la carpeta del proyecto a cualquier lado,</t>
+          <t>// POR QUE UN PARAMETRO Y NO UNA CONSULTA QUE LEA a UNA CELDA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="55" t="inlineStr">
         <is>
-          <t>// cambiar una sola celda y las cuatro consultas siguen funcionando.</t>
+          <t>// ----------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="55" t="inlineStr">
         <is>
-          <t>// Destino: Solo crear conexion (no se carga al modelo).</t>
+          <t>// La alternativa elegante seria leer la ruta desde una celda del libro con</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="55" t="inlineStr">
         <is>
-          <t>// ============================================================================</t>
+          <t>// Excel.CurrentWorkbook(). No se usa a proposito: Ventas quedaria referenciando</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="56" t="inlineStr">
-        <is>
-          <t>let</t>
+      <c r="B16" s="55" t="inlineStr">
+        <is>
+          <t>// otra consulta Y accediendo a un origen externo con File.Contents en el mismo</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // Excel.CurrentWorkbook lee rangos con nombre del libro que contiene la consulta</t>
+          <t>// paso, que es la condicion exacta que dispara el error</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TablaParametro = Excel.CurrentWorkbook(){[Name = "RutaDatos"]}[Content],</t>
+      <c r="B18" s="55" t="inlineStr">
+        <is>
+          <t>//</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="56" t="n"/>
+      <c r="B19" s="55" t="inlineStr">
+        <is>
+          <t>//     Formula.Firewall: la consulta 'Ventas' hace referencia a otras consultas</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="B20" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ValorCrudo = Table.FirstValue(TablaParametro, ""),</t>
+      <c r="B20" s="55" t="inlineStr">
+        <is>
+          <t>//     o pasos, por lo que puede que no tenga acceso directo a un origen de datos</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="56" t="n"/>
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t>//</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // Normaliza la barra final para poder concatenar el nombre de archivo sin riesgo</t>
+          <t>// Un parametro, en cambio, el motor lo resuelve como valor literal antes de</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    RutaNormalizada =</t>
+      <c r="B23" s="55" t="inlineStr">
+        <is>
+          <t>// evaluar la consulta, asi que no cuenta como referencia y el firewall no salta.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if Text.EndsWith(ValorCrudo, "\") then ValorCrudo</t>
+      <c r="B24" s="55" t="inlineStr">
+        <is>
+          <t>// Es la solucion idiomatica al problema, no un rodeo.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        else ValorCrudo &amp; "\"</t>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>//</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="56" t="inlineStr">
-        <is>
-          <t>in</t>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>// COMO SE CREA</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    RutaNormalizada</t>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t>// ----------------------------------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="55" t="inlineStr">
+        <is>
+          <t>// Opcion A (recomendada): Datos &gt; Obtener datos &gt; Iniciar el editor de Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="55" t="inlineStr">
+        <is>
+          <t>//   Query &gt; Inicio &gt; Administrar parametros &gt; Nuevo. Nombre: RutaDatos,</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="55" t="inlineStr">
         <is>
-          <t>// ============================================================================</t>
+          <t>//   Tipo: Texto, Valor actual: la ruta de la carpeta 'datos' terminada en \</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="55" t="inlineStr">
         <is>
-          <t>// Consulta: Ventas   (TABLA DE HECHOS)</t>
+          <t>//</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="55" t="inlineStr">
         <is>
-          <t>// ----------------------------------------------------------------------------</t>
+          <t>// Opcion B: crear una consulta en blanco, pegar la linea de abajo en el Editor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="55" t="inlineStr">
         <is>
-          <t>// Origen: ventas_historicas.csv (transaccional historico, delimitado por ";")</t>
+          <t>//   avanzado y renombrarla RutaDatos. El metadato IsParameterQuery hace que</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="55" t="inlineStr">
         <is>
-          <t>// Destino: Solo crear conexion + Agregar al Modelo de datos</t>
+          <t>//   Excel la trate como parametro, no como consulta.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="55" t="inlineStr">
         <is>
-          <t>//</t>
+          <t>// ============================================================================</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="55" t="inlineStr">
-        <is>
-          <t>// Los pasos estan renombrados a mano en el Editor Avanzado: en lugar de los</t>
-        </is>
-      </c>
+      <c r="B36" s="56" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="55" t="inlineStr">
-        <is>
-          <t>// #"Tipo cambiado", #"Filas filtradas1", #"Personalizada agregada2" que genera</t>
+      <c r="B37" s="56" t="inlineStr">
+        <is>
+          <t>"C:\Users\TU_USUARIO\Documents\ModeloBI\datos\"</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="55" t="inlineStr">
-        <is>
-          <t>// la interfaz, cada paso dice que hace. El orden tambien esta pensado: se filtra</t>
+      <c r="B38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    meta</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="55" t="inlineStr">
-        <is>
-          <t>// ANTES de calcular columnas, para no gastar CPU en filas que se van a descartar.</t>
+      <c r="B39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    [</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="55" t="inlineStr">
-        <is>
-          <t>// ============================================================================</t>
+      <c r="B40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        IsParameterQuery = true,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="56" t="inlineStr">
         <is>
-          <t>let</t>
+          <t xml:space="preserve">        List = null,</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    OrigenCSV = Csv.Document(</t>
+          <t xml:space="preserve">        DefaultValue = null,</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "ventas_historicas.csv"),</t>
+          <t xml:space="preserve">        Type = "Text",</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        [Delimiter = ";", Encoding = 65001, QuoteStyle = QuoteStyle.None]</t>
+          <t xml:space="preserve">        IsParameterQueryRequired = true</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="56" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    EncabezadosPromovidos = Table.PromoteHeaders(OrigenCSV, [PromoteAllScalars = true]),</t>
+          <t xml:space="preserve">    ]</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="56" t="n"/>
+      <c r="B48" s="55" t="inlineStr">
+        <is>
+          <t>// ============================================================================</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // --- 1. Tipado explicito -------------------------------------------------</t>
+          <t>// Consulta: Ventas   (TABLA DE HECHOS)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // Cultura "es-AR" para la fecha (dd/mm/aaaa) y "en-US" para los importes,</t>
+          <t>// ----------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // que en el CSV vienen con punto decimal. Sin esto Excel interpreta mal ambos.</t>
+          <t>// Origen: ventas_historicas.csv (transaccional historico, delimitado por ";")</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TiposCorregidos = Table.TransformColumnTypes(</t>
+      <c r="B52" s="55" t="inlineStr">
+        <is>
+          <t>// Destino: Solo crear conexion + Agregar al Modelo de datos</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        EncabezadosPromovidos,</t>
+      <c r="B53" s="55" t="inlineStr">
+        <is>
+          <t>//</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        {</t>
+      <c r="B54" s="55" t="inlineStr">
+        <is>
+          <t>// Los pasos estan renombrados a mano en el Editor Avanzado: en lugar de los</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"ID_Venta", type text},</t>
+      <c r="B55" s="55" t="inlineStr">
+        <is>
+          <t>// #"Tipo cambiado", #"Filas filtradas1", #"Personalizada agregada2" que genera</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"ID_Cliente", type text},</t>
+      <c r="B56" s="55" t="inlineStr">
+        <is>
+          <t>// la interfaz, cada paso dice que hace. El orden tambien esta pensado: se filtra</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"ID_Producto", type text},</t>
+      <c r="B57" s="55" t="inlineStr">
+        <is>
+          <t>// ANTES de calcular columnas, para no gastar CPU en filas que se van a descartar.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="B58" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Unidades", Int64.Type},</t>
+      <c r="B58" s="55" t="inlineStr">
+        <is>
+          <t>// ============================================================================</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"Descuento", type number},</t>
+          <t>let</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"Canal", type text},</t>
+          <t xml:space="preserve">    OrigenCSV = Csv.Document(</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"Estado", type text}</t>
+          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "ventas_historicas.csv"),</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">        [Delimiter = ";", Encoding = 65001, QuoteStyle = QuoteStyle.None]</t>
         </is>
       </c>
     </row>
@@ -2722,134 +2742,134 @@
       </c>
     </row>
     <row r="64">
-      <c r="B64" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FechasTipadas = Table.TransformColumnTypes(</t>
-        </is>
-      </c>
+      <c r="B64" s="56" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        TiposCorregidos, {{"Fecha", type date}}, "es-AR"</t>
+          <t xml:space="preserve">    EncabezadosPromovidos = Table.PromoteHeaders(OrigenCSV, [PromoteAllScalars = true]),</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="B66" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
-        </is>
-      </c>
+      <c r="B66" s="56" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ImportesTipados = Table.TransformColumnTypes(</t>
+      <c r="B67" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // --- 1. Tipado explicito -------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="B68" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        FechasTipadas,</t>
+      <c r="B68" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // Cultura "es-AR" para la fecha (dd/mm/aaaa) y "en-US" para los importes,</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="B69" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        {{"Precio_Unitario", type number}, {"Costo_Unitario", type number}},</t>
+      <c r="B69" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // que en el CSV vienen con punto decimal. Sin esto Excel interpreta mal ambos.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "en-US"</t>
+          <t xml:space="preserve">    TiposCorregidos = Table.TransformColumnTypes(</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t xml:space="preserve">        EncabezadosPromovidos,</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="B72" s="56" t="n"/>
+      <c r="B72" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        {</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="B73" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // --- 2. Limpieza de nulos y errores --------------------------------------</t>
+      <c r="B73" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"ID_Venta", type text},</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="B74" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // "n/d" en Precio_Unitario quedo como error tras el tipado: se elimina aca.</t>
+      <c r="B74" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"ID_Cliente", type text},</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SinErroresDeTipado = Table.RemoveRowsWithErrors(</t>
+          <t xml:space="preserve">            {"ID_Producto", type text},</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ImportesTipados, {"Precio_Unitario", "Costo_Unitario", "Fecha"}</t>
+          <t xml:space="preserve">            {"Unidades", Int64.Type},</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t xml:space="preserve">            {"Descuento", type number},</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="B78" s="56" t="n"/>
+      <c r="B78" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"Canal", type text},</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SinNulosCriticos = Table.SelectRows(</t>
+          <t xml:space="preserve">            {"Estado", type text}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        SinErroresDeTipado,</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        each [Unidades] &lt;&gt; null</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            and [ID_Cliente] &lt;&gt; null and [ID_Cliente] &lt;&gt; ""</t>
+          <t xml:space="preserve">    FechasTipadas = Table.TransformColumnTypes(</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            and [ID_Producto] &lt;&gt; null and [ID_Producto] &lt;&gt; ""</t>
+          <t xml:space="preserve">        TiposCorregidos, {{"Fecha", type date}}, "es-AR"</t>
         </is>
       </c>
     </row>
@@ -2861,33 +2881,37 @@
       </c>
     </row>
     <row r="85">
-      <c r="B85" s="56" t="n"/>
+      <c r="B85" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ImportesTipados = Table.TransformColumnTypes(</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="B86" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // --- 3. Filtrado estrategico ---------------------------------------------</t>
+      <c r="B86" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        FechasTipadas,</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="B87" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // ESTE es el paso renombrado que pide la consigna (la interfaz lo llamaba</t>
+      <c r="B87" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        {{"Precio_Unitario", type number}, {"Costo_Unitario", type number}},</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // #"Filas filtradas2"). Regla de negocio: las ventas anuladas no son ventas.</t>
+      <c r="B88" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        "en-US"</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    VentasFiltradas = Table.SelectRows(SinNulosCriticos, each [Estado] = "Confirmada"),</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
@@ -2897,548 +2921,548 @@
     <row r="91">
       <c r="B91" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // Duplicados exactos por ID_Venta: se conserva la primera ocurrencia</t>
+          <t xml:space="preserve">    // --- 2. Limpieza de nulos y errores --------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="B92" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    SinDuplicados = Table.Distinct(VentasFiltradas, {"ID_Venta"}),</t>
+      <c r="B92" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // "n/d" en Precio_Unitario quedo como error tras el tipado: se elimina aca.</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="B93" s="56" t="n"/>
+      <c r="B93" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    SinErroresDeTipado = Table.RemoveRowsWithErrors(</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="B94" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // --- 4. Estandarizacion de texto -----------------------------------------</t>
+      <c r="B94" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ImportesTipados, {"Precio_Unitario", "Costo_Unitario", "Fecha"}</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="B95" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // "online" / "ONLINE" / "Online" son el mismo canal: si no se unifica, la</t>
+      <c r="B95" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="B96" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // dimension se rompe y el grafico muestra tres barras donde deberia haber una.</t>
-        </is>
-      </c>
+      <c r="B96" s="56" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    CanalEstandarizado = Table.TransformColumns(</t>
+          <t xml:space="preserve">    SinNulosCriticos = Table.SelectRows(</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        SinDuplicados, {{"Canal", each Text.Proper(Text.Trim(_)), type text}}</t>
+          <t xml:space="preserve">        SinErroresDeTipado,</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t xml:space="preserve">        each [Unidades] &lt;&gt; null</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="B100" s="56" t="n"/>
+      <c r="B100" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            and [ID_Cliente] &lt;&gt; null and [ID_Cliente] &lt;&gt; ""</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="B101" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // --- 5. Columnas calculadas (solo sobre filas ya depuradas) --------------</t>
+      <c r="B101" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            and [ID_Producto] &lt;&gt; null and [ID_Producto] &lt;&gt; ""</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ConImporteBruto = Table.AddColumn(</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="B103" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        CanalEstandarizado, "Importe_Bruto",</t>
-        </is>
-      </c>
+      <c r="B103" s="56" t="n"/>
     </row>
     <row r="104">
-      <c r="B104" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        each [Unidades] * [Precio_Unitario], type number</t>
+      <c r="B104" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // --- 3. Filtrado estrategico ---------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="B105" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
+      <c r="B105" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // ESTE es el paso renombrado que pide la consigna (la interfaz lo llamaba</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="B106" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ConImporteNeto = Table.AddColumn(</t>
+      <c r="B106" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // #"Filas filtradas2"). Regla de negocio: las ventas anuladas no son ventas.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ConImporteBruto, "Importe_Neto",</t>
+          <t xml:space="preserve">    VentasFiltradas = Table.SelectRows(SinNulosCriticos, each [Estado] = "Confirmada"),</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="B108" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        each [Importe_Bruto] * (1 - [Descuento]), Currency.Type</t>
-        </is>
-      </c>
+      <c r="B108" s="56" t="n"/>
     </row>
     <row r="109">
-      <c r="B109" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
+      <c r="B109" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // Duplicados exactos por ID_Venta: se conserva la primera ocurrencia</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ConCostoTotal = Table.AddColumn(</t>
+          <t xml:space="preserve">    SinDuplicados = Table.Distinct(VentasFiltradas, {"ID_Venta"}),</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="B111" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ConImporteNeto, "Costo_Total",</t>
-        </is>
-      </c>
+      <c r="B111" s="56" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        each [Unidades] * [Costo_Unitario], Currency.Type</t>
+      <c r="B112" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // --- 4. Estandarizacion de texto -----------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="B113" s="56" t="inlineStr">
+      <c r="B113" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // "online" / "ONLINE" / "Online" son el mismo canal: si no se unifica, la</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // dimension se rompe y el grafico muestra tres barras donde deberia haber una.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    CanalEstandarizado = Table.TransformColumns(</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        SinDuplicados, {{"Canal", each Text.Proper(Text.Trim(_)), type text}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="B114" s="56" t="n"/>
-    </row>
-    <row r="115">
-      <c r="B115" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // --- 6. Reduccion del modelo ---------------------------------------------</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="B116" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Menos columnas = menos memoria en el motor xVelocity. Precio_Unitario y</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="B117" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Costo_Unitario ya estan absorbidos en las columnas de importe, y las</t>
-        </is>
-      </c>
-    </row>
     <row r="118">
-      <c r="B118" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // descriptivas (Cliente, Producto) viven en las dimensiones, no en los hechos.</t>
-        </is>
-      </c>
+      <c r="B118" s="56" t="n"/>
     </row>
     <row r="119">
-      <c r="B119" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    HechosFinales = Table.SelectColumns(</t>
+      <c r="B119" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // --- 5. Columnas calculadas (solo sobre filas ya depuradas) --------------</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="B120" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ConCostoTotal,</t>
+          <t xml:space="preserve">    ConImporteBruto = Table.AddColumn(</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="B121" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        CanalEstandarizado, "Importe_Bruto",</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="B122" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "ID_Venta", "Fecha", "ID_Cliente", "ID_Producto",</t>
+          <t xml:space="preserve">        each [Unidades] * [Precio_Unitario], type number</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="B123" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "Canal", "Unidades", "Importe_Bruto", "Importe_Neto", "Costo_Total"</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="B124" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">    ConImporteNeto = Table.AddColumn(</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="B125" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    )</t>
+          <t xml:space="preserve">        ConImporteBruto, "Importe_Neto",</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" s="56" t="inlineStr">
         <is>
-          <t>in</t>
+          <t xml:space="preserve">        each [Importe_Bruto] * (1 - [Descuento]), Currency.Type</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    HechosFinales</t>
+          <t xml:space="preserve">    ),</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ConCostoTotal = Table.AddColumn(</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConImporteNeto, "Costo_Total",</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="55" t="inlineStr">
-        <is>
-          <t>// ============================================================================</t>
+      <c r="B130" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        each [Unidades] * [Costo_Unitario], Currency.Type</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="B131" s="55" t="inlineStr">
-        <is>
-          <t>// LAS TRES DIMENSIONES DEL ESQUEMA EN ESTRELLA</t>
+      <c r="B131" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="B132" s="55" t="inlineStr">
-        <is>
-          <t>// Cada bloque es una consulta independiente. Copiar cada let...in por separado</t>
-        </is>
-      </c>
+      <c r="B132" s="56" t="n"/>
     </row>
     <row r="133">
       <c r="B133" s="55" t="inlineStr">
         <is>
-          <t>// en su propio Editor Avanzado.</t>
+          <t xml:space="preserve">    // --- 6. Reduccion del modelo ---------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="B134" s="55" t="inlineStr">
         <is>
-          <t>// Destino de las tres: Solo crear conexion + Agregar al Modelo de datos</t>
+          <t xml:space="preserve">    // Menos columnas = menos memoria en el motor xVelocity. Precio_Unitario y</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="B135" s="55" t="inlineStr">
         <is>
-          <t>// ============================================================================</t>
+          <t xml:space="preserve">    // Costo_Unitario ya estan absorbidos en las columnas de importe, y las</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="B136" s="56" t="n"/>
+      <c r="B136" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // descriptivas (Cliente, Producto) viven en las dimensiones, no en los hechos.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="B137" s="56" t="n"/>
+      <c r="B137" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    HechosFinales = Table.SelectColumns(</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="B138" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
+      <c r="B138" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConCostoTotal,</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="B139" s="55" t="inlineStr">
-        <is>
-          <t>// Consulta: Clientes        Origen: maestras.xlsx, tabla tbl_Clientes</t>
+      <c r="B139" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="B140" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
+      <c r="B140" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            "ID_Venta", "Fecha", "ID_Cliente", "ID_Producto",</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" s="56" t="inlineStr">
         <is>
-          <t>let</t>
+          <t xml:space="preserve">            "Canal", "Unidades", "Importe_Bruto", "Importe_Neto", "Costo_Total"</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    LibroMaestras = Excel.Workbook(</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "maestras.xlsx"), null, true</t>
+          <t xml:space="preserve">    )</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t>in</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="B145" s="56" t="n"/>
-    </row>
-    <row r="146">
-      <c r="B146" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Se toma la TABLA con nombre, no la hoja: si alguien inserta filas arriba</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="B147" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // la consulta no se rompe, cosa que si pasa al apuntar a la hoja entera.</t>
+      <c r="B145" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    HechosFinales</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="B148" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TablaClientes = LibroMaestras{[Item = "tbl_Clientes", Kind = "Table"]}[Data],</t>
+      <c r="B148" s="55" t="inlineStr">
+        <is>
+          <t>// ============================================================================</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="B149" s="56" t="n"/>
+      <c r="B149" s="55" t="inlineStr">
+        <is>
+          <t>// LAS TRES DIMENSIONES DEL ESQUEMA EN ESTRELLA</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="B150" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TiposClientes = Table.TransformColumnTypes(</t>
+      <c r="B150" s="55" t="inlineStr">
+        <is>
+          <t>// Cada bloque es una consulta independiente. Copiar cada let...in por separado</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="B151" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        TablaClientes,</t>
+      <c r="B151" s="55" t="inlineStr">
+        <is>
+          <t>// en su propio Editor Avanzado.</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="B152" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        {</t>
+      <c r="B152" s="55" t="inlineStr">
+        <is>
+          <t>// Destino de las tres: Solo crear conexion + Agregar al Modelo de datos</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="B153" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"ID_Cliente", type text},</t>
+      <c r="B153" s="55" t="inlineStr">
+        <is>
+          <t>// ============================================================================</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="B154" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Cliente", type text},</t>
-        </is>
-      </c>
+      <c r="B154" s="56" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Region", type text},</t>
-        </is>
-      </c>
+      <c r="B155" s="56" t="n"/>
     </row>
     <row r="156">
-      <c r="B156" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Segmento", type text},</t>
+      <c r="B156" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="B157" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Antiguedad_Anios", Int64.Type}</t>
+      <c r="B157" s="55" t="inlineStr">
+        <is>
+          <t>// Consulta: Clientes        Origen: maestras.xlsx, tabla tbl_Clientes</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="B158" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        }</t>
+      <c r="B158" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" s="56" t="inlineStr">
         <is>
+          <t>let</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LibroMaestras = Excel.Workbook(</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "maestras.xlsx"), null, true</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" s="56" t="inlineStr">
+        <is>
           <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="B160" s="56" t="n"/>
-    </row>
-    <row r="161">
-      <c r="B161" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // La clave primaria no admite nulos ni repetidos: si los tuviera, la</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="B162" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // relacion 1:N contra la tabla de hechos fallaria al crearse.</t>
-        </is>
-      </c>
-    </row>
     <row r="163">
-      <c r="B163" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ClavesValidas = Table.SelectRows(</t>
-        </is>
-      </c>
+      <c r="B163" s="56" t="n"/>
     </row>
     <row r="164">
-      <c r="B164" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        TiposClientes, each [ID_Cliente] &lt;&gt; null and [ID_Cliente] &lt;&gt; ""</t>
+      <c r="B164" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // Se toma la TABLA con nombre, no la hoja: si alguien inserta filas arriba</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="B165" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
+      <c r="B165" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // la consulta no se rompe, cosa que si pasa al apuntar a la hoja entera.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="B166" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DimClientes = Table.Distinct(ClavesValidas, {"ID_Cliente"})</t>
+          <t xml:space="preserve">    TablaClientes = LibroMaestras{[Item = "tbl_Clientes", Kind = "Table"]}[Data],</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="B167" s="56" t="inlineStr">
-        <is>
-          <t>in</t>
-        </is>
-      </c>
+      <c r="B167" s="56" t="n"/>
     </row>
     <row r="168">
       <c r="B168" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DimClientes</t>
+          <t xml:space="preserve">    TiposClientes = Table.TransformColumnTypes(</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="B169" s="56" t="n"/>
+      <c r="B169" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        TablaClientes,</t>
+        </is>
+      </c>
     </row>
     <row r="170">
-      <c r="B170" s="56" t="n"/>
+      <c r="B170" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        {</t>
+        </is>
+      </c>
     </row>
     <row r="171">
-      <c r="B171" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
+      <c r="B171" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"ID_Cliente", type text},</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="B172" s="55" t="inlineStr">
-        <is>
-          <t>// Consulta: Productos       Origen: maestras.xlsx, tabla tbl_Productos</t>
+      <c r="B172" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"Cliente", type text},</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="B173" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
+      <c r="B173" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"Region", type text},</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="B174" s="56" t="inlineStr">
         <is>
-          <t>let</t>
+          <t xml:space="preserve">            {"Segmento", type text},</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="B175" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    LibroMaestras = Excel.Workbook(</t>
+          <t xml:space="preserve">            {"Antiguedad_Anios", Int64.Type}</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="B176" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "maestras.xlsx"), null, true</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
@@ -3453,106 +3477,106 @@
       <c r="B178" s="56" t="n"/>
     </row>
     <row r="179">
-      <c r="B179" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    TablaProductos = LibroMaestras{[Item = "tbl_Productos", Kind = "Table"]}[Data],</t>
+      <c r="B179" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // La clave primaria no admite nulos ni repetidos: si los tuviera, la</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="B180" s="56" t="n"/>
+      <c r="B180" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // relacion 1:N contra la tabla de hechos fallaria al crearse.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="B181" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    TiposProductos = Table.TransformColumnTypes(</t>
+          <t xml:space="preserve">    ClavesValidas = Table.SelectRows(</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="B182" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        TablaProductos,</t>
+          <t xml:space="preserve">        TiposClientes, each [ID_Cliente] &lt;&gt; null and [ID_Cliente] &lt;&gt; ""</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="B183" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="B184" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"ID_Producto", type text},</t>
+          <t xml:space="preserve">    DimClientes = Table.Distinct(ClavesValidas, {"ID_Cliente"})</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="B185" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"Producto", type text},</t>
+          <t>in</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="B186" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">            {"Categoria", type text},</t>
+          <t xml:space="preserve">    DimClientes</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="B187" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Subcategoria", type text},</t>
-        </is>
-      </c>
+      <c r="B187" s="56" t="n"/>
     </row>
     <row r="188">
-      <c r="B188" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Costo_Unitario", Currency.Type},</t>
-        </is>
-      </c>
+      <c r="B188" s="56" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            {"Precio_Lista", Currency.Type}</t>
+      <c r="B189" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="B190" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        }</t>
+      <c r="B190" s="55" t="inlineStr">
+        <is>
+          <t>// Consulta: Productos       Origen: maestras.xlsx, tabla tbl_Productos</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="B191" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
+      <c r="B191" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="B192" s="56" t="n"/>
+      <c r="B192" s="56" t="inlineStr">
+        <is>
+          <t>let</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="B193" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ClavesValidas = Table.SelectRows(</t>
+          <t xml:space="preserve">    LibroMaestras = Excel.Workbook(</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="B194" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        TiposProductos, each [ID_Producto] &lt;&gt; null and [ID_Producto] &lt;&gt; ""</t>
+          <t xml:space="preserve">        File.Contents(RutaDatos &amp; "maestras.xlsx"), null, true</t>
         </is>
       </c>
     </row>
@@ -3567,314 +3591,310 @@
       <c r="B196" s="56" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Columna de apoyo para ordenar y agrupar el margen teorico por producto</t>
+      <c r="B197" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    TablaProductos = LibroMaestras{[Item = "tbl_Productos", Kind = "Table"]}[Data],</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="B198" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ConMargenLista = Table.AddColumn(</t>
-        </is>
-      </c>
+      <c r="B198" s="56" t="n"/>
     </row>
     <row r="199">
       <c r="B199" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ClavesValidas, "Margen_Lista_Pct",</t>
+          <t xml:space="preserve">    TiposProductos = Table.TransformColumnTypes(</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="B200" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        each if [Precio_Lista] = 0 then null</t>
+          <t xml:space="preserve">        TablaProductos,</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="B201" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">             else ([Precio_Lista] - [Costo_Unitario]) / [Precio_Lista],</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="B202" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Percentage.Type</t>
+          <t xml:space="preserve">            {"ID_Producto", type text},</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="B203" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t xml:space="preserve">            {"Producto", type text},</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="B204" s="56" t="n"/>
+      <c r="B204" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            {"Categoria", type text},</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="B205" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DimProductos = Table.Distinct(ConMargenLista, {"ID_Producto"})</t>
+          <t xml:space="preserve">            {"Subcategoria", type text},</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="B206" s="56" t="inlineStr">
         <is>
-          <t>in</t>
+          <t xml:space="preserve">            {"Costo_Unitario", Currency.Type},</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="B207" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DimProductos</t>
+          <t xml:space="preserve">            {"Precio_Lista", Currency.Type}</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="B208" s="56" t="n"/>
+      <c r="B208" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
     </row>
     <row r="209">
-      <c r="B209" s="56" t="n"/>
+      <c r="B209" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
+        </is>
+      </c>
     </row>
     <row r="210">
-      <c r="B210" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
-        </is>
-      </c>
+      <c r="B210" s="56" t="n"/>
     </row>
     <row r="211">
-      <c r="B211" s="55" t="inlineStr">
-        <is>
-          <t>// Consulta: Calendario      Origen: NINGUNO - generada 100% en lenguaje M</t>
+      <c r="B211" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ClavesValidas = Table.SelectRows(</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="B212" s="55" t="inlineStr">
-        <is>
-          <t>// ----------------------------------------------------------------------------</t>
+      <c r="B212" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        TiposProductos, each [ID_Producto] &lt;&gt; null and [ID_Producto] &lt;&gt; ""</t>
         </is>
       </c>
     </row>
     <row r="213">
-      <c r="B213" s="55" t="inlineStr">
-        <is>
-          <t>// No hay archivo detras de esta tabla: se construye con List.Dates a partir del</t>
+      <c r="B213" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="214">
-      <c r="B214" s="55" t="inlineStr">
-        <is>
-          <t>// rango real de fechas de la tabla de hechos. Si manana llegan ventas de 2027,</t>
-        </is>
-      </c>
+      <c r="B214" s="56" t="n"/>
     </row>
     <row r="215">
       <c r="B215" s="55" t="inlineStr">
         <is>
-          <t>// el calendario se extiende solo al actualizar. Es el ejemplo mas claro de por</t>
+          <t xml:space="preserve">    // Columna de apoyo para ordenar y agrupar el margen teorico por producto</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="B216" s="55" t="inlineStr">
-        <is>
-          <t>// que conviene escribir M a mano en vez de depender de los botones.</t>
+      <c r="B216" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ConMargenLista = Table.AddColumn(</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="B217" s="55" t="inlineStr">
-        <is>
-          <t>// ############################################################################</t>
+      <c r="B217" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ClavesValidas, "Margen_Lista_Pct",</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="B218" s="56" t="inlineStr">
         <is>
-          <t>let</t>
+          <t xml:space="preserve">        each if [Precio_Lista] = 0 then null</t>
         </is>
       </c>
     </row>
     <row r="219">
-      <c r="B219" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Se leen los limites reales desde Ventas para no fijar fechas a mano</t>
+      <c r="B219" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             else ([Precio_Lista] - [Costo_Unitario]) / [Precio_Lista],</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="B220" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FechaMinima = Date.StartOfYear(List.Min(Ventas[Fecha])),</t>
+          <t xml:space="preserve">        Percentage.Type</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="B221" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FechaMaxima = Date.EndOfYear(List.Max(Ventas[Fecha])),</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="222">
-      <c r="B222" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    CantidadDias = Duration.Days(FechaMaxima - FechaMinima) + 1,</t>
-        </is>
-      </c>
+      <c r="B222" s="56" t="n"/>
     </row>
     <row r="223">
-      <c r="B223" s="56" t="n"/>
+      <c r="B223" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DimProductos = Table.Distinct(ConMargenLista, {"ID_Producto"})</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="B224" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ListaFechas = List.Dates(FechaMinima, CantidadDias, #duration(1, 0, 0, 0)),</t>
+          <t>in</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="B225" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    TablaBase = Table.FromList(</t>
+          <t xml:space="preserve">    DimProductos</t>
         </is>
       </c>
     </row>
     <row r="226">
-      <c r="B226" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ListaFechas, Splitter.SplitByNothing(), {"Fecha"}, null, ExtraValues.Error</t>
-        </is>
-      </c>
+      <c r="B226" s="56" t="n"/>
     </row>
     <row r="227">
-      <c r="B227" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
-        </is>
-      </c>
+      <c r="B227" s="56" t="n"/>
     </row>
     <row r="228">
-      <c r="B228" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FechaTipada = Table.TransformColumnTypes(TablaBase, {{"Fecha", type date}}),</t>
+      <c r="B228" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="B229" s="56" t="n"/>
+      <c r="B229" s="55" t="inlineStr">
+        <is>
+          <t>// Consulta: Calendario      Origen: NINGUNO - generada 100% en lenguaje M</t>
+        </is>
+      </c>
     </row>
     <row r="230">
-      <c r="B230" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ConAnio = Table.AddColumn(FechaTipada, "Anio", each Date.Year([Fecha]), Int64.Type),</t>
+      <c r="B230" s="55" t="inlineStr">
+        <is>
+          <t>// ----------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="231">
-      <c r="B231" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ConTrimestre = Table.AddColumn(</t>
+      <c r="B231" s="55" t="inlineStr">
+        <is>
+          <t>// No hay archivo detras de esta tabla: se construye con List.Dates a partir del</t>
         </is>
       </c>
     </row>
     <row r="232">
-      <c r="B232" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ConAnio, "Trimestre", each "T" &amp; Text.From(Date.QuarterOfYear([Fecha])), type text</t>
+      <c r="B232" s="55" t="inlineStr">
+        <is>
+          <t>// rango real de fechas de la tabla de hechos. Si manana llegan ventas de 2027,</t>
         </is>
       </c>
     </row>
     <row r="233">
-      <c r="B233" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
+      <c r="B233" s="55" t="inlineStr">
+        <is>
+          <t>// el calendario se extiende solo al actualizar. Es el ejemplo mas claro de por</t>
         </is>
       </c>
     </row>
     <row r="234">
-      <c r="B234" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ConMes = Table.AddColumn(ConTrimestre, "Mes", each Date.Month([Fecha]), Int64.Type),</t>
+      <c r="B234" s="55" t="inlineStr">
+        <is>
+          <t>// que conviene escribir M a mano en vez de depender de los botones.</t>
         </is>
       </c>
     </row>
     <row r="235">
-      <c r="B235" s="56" t="n"/>
+      <c r="B235" s="55" t="inlineStr">
+        <is>
+          <t>// ############################################################################</t>
+        </is>
+      </c>
     </row>
     <row r="236">
-      <c r="B236" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    // Nombre de mes forzado a es-AR: sin la cultura, el idioma depende de la</t>
+      <c r="B236" s="56" t="inlineStr">
+        <is>
+          <t>let</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="B237" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    // maquina que actualice y el reporte alterna entre "enero" y "January".</t>
+          <t xml:space="preserve">    // Se leen los limites reales desde Ventas para no fijar fechas a mano</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="B238" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ConNombreMes = Table.AddColumn(</t>
+          <t xml:space="preserve">    FechaMinima = Date.StartOfYear(List.Min(Ventas[Fecha])),</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="B239" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ConMes, "Nombre_Mes",</t>
+          <t xml:space="preserve">    FechaMaxima = Date.EndOfYear(List.Max(Ventas[Fecha])),</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="B240" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        each Text.Proper(Date.ToText([Fecha], "MMMM", "es-AR")), type text</t>
+          <t xml:space="preserve">    CantidadDias = Duration.Days(FechaMaxima - FechaMinima) + 1,</t>
         </is>
       </c>
     </row>
     <row r="241">
-      <c r="B241" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ),</t>
-        </is>
-      </c>
+      <c r="B241" s="56" t="n"/>
     </row>
     <row r="242">
       <c r="B242" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ConAnioMes = Table.AddColumn(</t>
+          <t xml:space="preserve">    ListaFechas = List.Dates(FechaMinima, CantidadDias, #duration(1, 0, 0, 0)),</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="B243" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ConNombreMes, "Anio_Mes",</t>
+          <t xml:space="preserve">    TablaBase = Table.FromList(</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="B244" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        each Text.From([Anio]) &amp; "-" &amp; Text.PadStart(Text.From([Mes]), 2, "0"), type text</t>
+          <t xml:space="preserve">        ListaFechas, Splitter.SplitByNothing(), {"Fecha"}, null, ExtraValues.Error</t>
         </is>
       </c>
     </row>
@@ -3888,68 +3908,186 @@
     <row r="246">
       <c r="B246" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ConDiaSemana = Table.AddColumn(</t>
+          <t xml:space="preserve">    FechaTipada = Table.TransformColumnTypes(TablaBase, {{"Fecha", type date}}),</t>
         </is>
       </c>
     </row>
     <row r="247">
-      <c r="B247" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ConAnioMes, "Dia_Semana",</t>
-        </is>
-      </c>
+      <c r="B247" s="56" t="n"/>
     </row>
     <row r="248">
       <c r="B248" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        each Text.Proper(Date.ToText([Fecha], "dddd", "es-AR")), type text</t>
+          <t xml:space="preserve">    ConAnio = Table.AddColumn(FechaTipada, "Anio", each Date.Year([Fecha]), Int64.Type),</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="B249" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ),</t>
+          <t xml:space="preserve">    ConTrimestre = Table.AddColumn(</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="B250" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DimCalendario = Table.AddColumn(</t>
+          <t xml:space="preserve">        ConAnio, "Trimestre", each "T" &amp; Text.From(Date.QuarterOfYear([Fecha])), type text</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="B251" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ConDiaSemana, "Es_Fin_De_Semana",</t>
+          <t xml:space="preserve">    ),</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="B252" s="56" t="inlineStr">
         <is>
+          <t xml:space="preserve">    ConMes = Table.AddColumn(ConTrimestre, "Mes", each Date.Month([Fecha]), Int64.Type),</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="B253" s="56" t="n"/>
+    </row>
+    <row r="254">
+      <c r="B254" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // Nombre de mes forzado a es-AR: sin la cultura, el idioma depende de la</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="B255" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    // maquina que actualice y el reporte alterna entre "enero" y "January".</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="B256" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ConNombreMes = Table.AddColumn(</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="B257" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConMes, "Nombre_Mes",</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="B258" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        each Text.Proper(Date.ToText([Fecha], "MMMM", "es-AR")), type text</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="B259" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="B260" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ConAnioMes = Table.AddColumn(</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="B261" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConNombreMes, "Anio_Mes",</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="B262" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        each Text.From([Anio]) &amp; "-" &amp; Text.PadStart(Text.From([Mes]), 2, "0"), type text</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="B263" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="B264" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ConDiaSemana = Table.AddColumn(</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="B265" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConAnioMes, "Dia_Semana",</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="B266" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        each Text.Proper(Date.ToText([Fecha], "dddd", "es-AR")), type text</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="B267" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ),</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="B268" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    DimCalendario = Table.AddColumn(</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="B269" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ConDiaSemana, "Es_Fin_De_Semana",</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="B270" s="56" t="inlineStr">
+        <is>
           <t xml:space="preserve">        each Date.DayOfWeek([Fecha], Day.Monday) &gt;= 5, type logical</t>
         </is>
       </c>
     </row>
-    <row r="253">
-      <c r="B253" s="56" t="inlineStr">
+    <row r="271">
+      <c r="B271" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">    )</t>
         </is>
       </c>
     </row>
-    <row r="254">
-      <c r="B254" s="56" t="inlineStr">
+    <row r="272">
+      <c r="B272" s="56" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
     </row>
-    <row r="255">
-      <c r="B255" s="56" t="inlineStr">
+    <row r="273">
+      <c r="B273" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">    DimCalendario</t>
         </is>
@@ -4684,7 +4822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C43"/>
+  <dimension ref="B2:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4714,261 +4852,296 @@
       </c>
       <c r="C5" s="58" t="inlineStr">
         <is>
-          <t>PONER LA RUTA DE DATOS</t>
+          <t>CREAR EL PARAMETRO DE RUTA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>Hoja Config, celda B3: pegar la ruta de la carpeta 'datos' de este proyecto.</t>
+          <t>Dejar el .xlsx en una carpeta y el CSV + maestras.xlsx en una subcarpeta</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="C7" s="59" t="inlineStr">
         <is>
-          <t>Tiene que terminar en barra invertida. Ya viene con la ruta con la que se genero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="57" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C9" s="58" t="inlineStr">
-        <is>
-          <t>CREAR LAS 5 CONSULTAS DE POWER QUERY</t>
+          <t>llamada 'datos'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>Datos &gt; Obtener datos &gt; Iniciar el editor de Power Query.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="59" t="inlineStr">
+        <is>
+          <t>Inicio &gt; Administrar parametros &gt; Nuevo:</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="C10" s="59" t="inlineStr">
         <is>
-          <t>Datos &gt; Obtener datos &gt; De otras fuentes &gt; Consulta en blanco.</t>
+          <t xml:space="preserve">   Nombre: RutaDatos     Tipo: Texto</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="C11" s="59" t="inlineStr">
         <is>
-          <t>En cada consulta: Inicio &gt; Editor avanzado, borrar todo y pegar el bloque</t>
+          <t xml:space="preserve">   Valor actual: la ruta de esa carpeta 'datos', TERMINADA EN \</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="C12" s="59" t="inlineStr">
         <is>
-          <t>correspondiente de la hoja Anexo_Codigo_M. Renombrar la consulta con el</t>
+          <t xml:space="preserve">   ejemplo:  C:\Users\Lleyton\Documents\ModeloBI\datos\</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="C13" s="59" t="inlineStr">
         <is>
-          <t>nombre exacto del encabezado del bloque.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="59" t="inlineStr">
-        <is>
-          <t>Orden obligatorio: RutaDatos, Ventas, Clientes, Productos, Calendario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="C15" s="59" t="inlineStr">
-        <is>
-          <t>(Calendario lee de Ventas, asi que Ventas tiene que existir antes.)</t>
+          <t>La celda B3 de la hoja Config tiene ese mismo valor para copiarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="57" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="inlineStr">
+        <is>
+          <t>CREAR LAS 4 CONSULTAS DE POWER QUERY</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="C16" s="59" t="inlineStr">
         <is>
-          <t>En RutaDatos: clic derecho &gt; Cargar en... &gt; Solo crear conexion.</t>
+          <t>En el editor: Inicio &gt; Nuevos orígenes &gt; Consulta en blanco.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="C17" s="59" t="inlineStr">
         <is>
-          <t>En las otras cuatro: Cargar en... &gt; Solo crear conexion + tildar</t>
+          <t>En cada consulta: Inicio &gt; Editor avanzado, borrar todo y pegar el bloque</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="C18" s="59" t="inlineStr">
         <is>
-          <t>'Agregar estos datos al Modelo de datos'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="57" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C20" s="58" t="inlineStr">
-        <is>
-          <t>ARMAR EL ESQUEMA EN ESTRELLA</t>
+          <t>correspondiente de la hoja Anexo_Codigo_M. Renombrar la consulta con el</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>nombre exacto del encabezado del bloque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>Orden obligatorio: Ventas, Clientes, Productos, Calendario.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="C21" s="59" t="inlineStr">
         <is>
-          <t>Power Pivot &gt; Administrar &gt; Vista de diagrama.</t>
+          <t>(Calendario lee de Ventas, asi que Ventas tiene que existir antes.)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="C22" s="59" t="inlineStr">
         <is>
-          <t>Ubicar Ventas en el centro y las tres dimensiones alrededor.</t>
+          <t>En las cuatro: Cargar en... &gt; Solo crear conexion + tildar</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="C23" s="59" t="inlineStr">
         <is>
-          <t>Arrastrar Clientes[ID_Cliente] sobre Ventas[ID_Cliente].</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="59" t="inlineStr">
-        <is>
-          <t>Arrastrar Productos[ID_Producto] sobre Ventas[ID_Producto].</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="59" t="inlineStr">
-        <is>
-          <t>Arrastrar Calendario[Fecha] sobre Ventas[Fecha].</t>
+          <t>'Agregar estos datos al Modelo de datos'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="57" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C25" s="58" t="inlineStr">
+        <is>
+          <t>ARMAR EL ESQUEMA EN ESTRELLA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="59" t="inlineStr">
         <is>
-          <t>Verificar que el '1' quede del lado de la dimension y el '*' del lado de Ventas.</t>
+          <t>Power Pivot &gt; Administrar &gt; Vista de diagrama.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="C27" s="59" t="inlineStr">
         <is>
-          <t>Seleccionar Calendario &gt; Disenio &gt; Marcar como tabla de fechas &gt; Fecha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="57" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C29" s="58" t="inlineStr">
-        <is>
-          <t>CARGAR LAS MEDIDAS DAX</t>
+          <t>Ubicar Ventas en el centro y las tres dimensiones alrededor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" s="59" t="inlineStr">
+        <is>
+          <t>Arrastrar Clientes[ID_Cliente] sobre Ventas[ID_Cliente].</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="59" t="inlineStr">
+        <is>
+          <t>Arrastrar Productos[ID_Producto] sobre Ventas[ID_Producto].</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="59" t="inlineStr">
         <is>
-          <t>Power Pivot &gt; Medidas &gt; Nueva medida, con la tabla Ventas seleccionada.</t>
+          <t>Arrastrar Calendario[Fecha] sobre Ventas[Fecha].</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="59" t="inlineStr">
         <is>
-          <t>Crear las 7 medidas de la hoja Anexo_Medidas_DAX, en ese orden</t>
+          <t>Verificar que el '1' quede del lado de la dimension y el '*' del lado de Ventas.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="C32" s="59" t="inlineStr">
         <is>
-          <t>(las ultimas dependen de las primeras).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="C33" s="59" t="inlineStr">
-        <is>
-          <t>Nombre de la medida y formato estan indicados arriba de cada formula.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="57" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C35" s="58" t="inlineStr">
-        <is>
-          <t>VERIFICAR LA SIMULACION</t>
+          <t>Seleccionar Calendario &gt; Disenio &gt; Marcar como tabla de fechas &gt; Fecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="57" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="inlineStr">
+        <is>
+          <t>CARGAR LAS MEDIDAS DAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>Power Pivot &gt; Medidas &gt; Nueva medida, con la tabla Ventas seleccionada.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="C36" s="59" t="inlineStr">
         <is>
-          <t>Los tres escenarios ya estan guardados en el libro: Datos &gt; Analisis de</t>
+          <t>Crear las 7 medidas de la hoja Anexo_Medidas_DAX, en ese orden</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="C37" s="59" t="inlineStr">
         <is>
-          <t>hipotesis &gt; Administrador de escenarios y aparecen Pesimista, Base y Optimista.</t>
+          <t>(las ultimas dependen de las primeras).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="C38" s="59" t="inlineStr">
         <is>
-          <t>Buscar objetivo: celda C24, valor de C28, cambiando C10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="C39" s="59" t="inlineStr">
-        <is>
-          <t>Tiene que dar 9.181 unidades aprox. Deshacer con Ctrl+Z despues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="57" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C41" s="58" t="inlineStr">
-        <is>
-          <t>GUARDAR</t>
+          <t>Nombre de la medida y formato estan indicados arriba de cada formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="57" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C40" s="58" t="inlineStr">
+        <is>
+          <t>VERIFICAR LA SIMULACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" s="59" t="inlineStr">
+        <is>
+          <t>Los tres escenarios ya estan guardados en el libro: Datos &gt; Analisis de</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="C42" s="59" t="inlineStr">
         <is>
-          <t>Guardar como .xlsx manteniendo el nombre PreEntrega_ModeloBI_MurphyLleyton.</t>
+          <t>hipotesis &gt; Administrador de escenarios y aparecen Pesimista, Base y Optimista.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>Buscar objetivo: celda C24, valor de C28, cambiando C10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="59" t="inlineStr">
+        <is>
+          <t>Tiene que dar 9.181 unidades aprox. Deshacer con Ctrl+Z despues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="B46" s="57" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C46" s="58" t="inlineStr">
+        <is>
+          <t>GUARDAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="59" t="inlineStr">
+        <is>
+          <t>Guardar como .xlsx manteniendo el nombre PreEntrega_ModeloBI_MurphyLleyton.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="59" t="inlineStr">
         <is>
           <t>Al guardar, el modelo de Power Pivot y las consultas quedan dentro del archivo.</t>
         </is>

</xml_diff>